<commit_message>
up to b0bc3a2 plus yourquest change
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="414">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -1330,6 +1330,12 @@
   </si>
   <si>
     <t xml:space="preserve">shows/hides the events of the background profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload2RoastHubs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload current loaded profile to RoastHubs</t>
   </si>
   <si>
     <t xml:space="preserve">RC Command</t>
@@ -2179,7 +2185,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C170"/>
+  <dimension ref="A1:C171"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -3388,17 +3394,17 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="1" t="s">
+      <c r="B149" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="B149" s="3" t="s">
+      <c r="C149" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="C149" s="1" t="s">
+    </row>
+    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="1" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="3" t="s">
         <v>381</v>
       </c>
@@ -3456,15 +3462,15 @@
     </row>
     <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="3" t="s">
-        <v>244</v>
+        <v>395</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
-        <v>396</v>
+        <v>244</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>397</v>
@@ -3480,26 +3486,26 @@
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B161" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C160" s="1" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="B161" s="3" t="s">
-        <v>393</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="B162" s="3" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>404</v>
@@ -3507,69 +3513,77 @@
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3" t="s">
-        <v>383</v>
+        <v>405</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="1" t="s">
-        <v>406</v>
-      </c>
       <c r="B164" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B165" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C164" s="1" t="s">
+      <c r="C165" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B165" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>131</v>
+        <v>409</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>132</v>
+        <v>410</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>409</v>
+        <v>134</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>138</v>
+        <v>411</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="3" t="s">
-        <v>410</v>
+        <v>137</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>411</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B171" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
up to 1604ca5, more lc
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$135</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$140</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="424">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -997,6 +997,36 @@
   </si>
   <si>
     <t xml:space="preserve">sets the beta and gamma parameters of the PID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidDerivativeFilter(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets derivative filter size;  0 &lt;= n &lt; 6 (n:int)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidDerivativeLimit(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets derivative limit (Dlimit); n &gt;= 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidILF(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets integral limit factor; 0&lt;=n&lt;=1 (n:float)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidIWP(&lt;bool&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggles integral windup prevention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidIRoC(&lt;bool&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggles integral reset on target</t>
   </si>
   <si>
     <t xml:space="preserve">adjustSV(&lt;float&gt;)</t>
@@ -2185,7 +2215,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C171"/>
+  <dimension ref="A1:C176"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -3211,66 +3241,66 @@
     </row>
     <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3" t="s">
-        <v>133</v>
+        <v>335</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="3" t="s">
-        <v>137</v>
+        <v>339</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>138</v>
+        <v>340</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3" t="s">
-        <v>342</v>
+        <v>133</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3" t="s">
-        <v>346</v>
+        <v>137</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>347</v>
+        <v>138</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,49 +3432,49 @@
       </c>
     </row>
     <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="1" t="s">
+      <c r="B150" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="B150" s="3" t="s">
+      <c r="C150" s="1" t="s">
         <v>381</v>
-      </c>
-      <c r="C150" s="1" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C151" s="1" t="s">
         <v>383</v>
-      </c>
-      <c r="C151" s="1" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="C152" s="1" t="s">
         <v>385</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>387</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C154" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="C154" s="1" t="s">
+    </row>
+    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="1" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="3" t="s">
         <v>391</v>
       </c>
@@ -3470,120 +3500,160 @@
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
-        <v>244</v>
+        <v>397</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="3" t="s">
-        <v>253</v>
+        <v>403</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="1" t="s">
-        <v>403</v>
-      </c>
       <c r="B162" s="3" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3" t="s">
-        <v>405</v>
+        <v>244</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="3" t="s">
-        <v>385</v>
+        <v>408</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="1" t="s">
-        <v>408</v>
-      </c>
       <c r="B165" s="3" t="s">
-        <v>129</v>
+        <v>410</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>130</v>
+        <v>411</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>409</v>
+        <v>253</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="s">
+        <v>413</v>
+      </c>
       <c r="B167" s="3" t="s">
-        <v>131</v>
+        <v>405</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>132</v>
+        <v>414</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>133</v>
+        <v>415</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>134</v>
+        <v>416</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>135</v>
+        <v>395</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="s">
+        <v>418</v>
+      </c>
       <c r="B170" s="3" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="3" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>413</v>
+        <v>420</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B172" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C172" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B173" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B174" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C174" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B175" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B176" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>